<commit_message>
Add Extras, update Mobiliario, add Notes section
</commit_message>
<xml_diff>
--- a/venuedata.xlsx
+++ b/venuedata.xlsx
@@ -23,12 +23,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="48">
   <si>
     <t xml:space="preserve">  Inspace  -  15 de octubre</t>
   </si>
   <si>
-    <t xml:space="preserve">  Solo modifica los valores en la columna PRECIO (azul). No cambies otras columnas.</t>
+    <t xml:space="preserve">  Solo modifica los valores en la columna PRECIO (azul) y el campo de NOTAS al final.</t>
   </si>
   <si>
     <t xml:space="preserve">Categoria</t>
@@ -112,16 +112,25 @@
     <t xml:space="preserve">Mobiliario</t>
   </si>
   <si>
-    <t xml:space="preserve">Mesas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sillas / lounge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Podios / atril</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Otros muebles</t>
+    <t xml:space="preserve">Sillas y mesas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stands</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decoracion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">extras</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extras</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valet Parking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuente electrica</t>
   </si>
   <si>
     <t xml:space="preserve">catering</t>
@@ -142,7 +151,13 @@
     <t xml:space="preserve">TOTAL ESTIMADO  (sin catering)</t>
   </si>
   <si>
-    <t xml:space="preserve">  * El catering se selecciona en la pagina web. Ingresa el precio de cada opcion en las filas de Catering.</t>
+    <t xml:space="preserve">  * El catering se selecciona en la pagina web. Ingresa el precio de cada opcion arriba.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  NOTAS / COMENTARIOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">notas</t>
   </si>
   <si>
     <t xml:space="preserve">  Camino Real  -  15 de octubre</t>
@@ -162,7 +177,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -270,8 +285,15 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -306,6 +328,24 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF8E6"/>
         <bgColor rgb="FFFFF9E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4A6741"/>
+        <bgColor rgb="FF555555"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF3A5A7A"/>
+        <bgColor rgb="FF1F5C8B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF0F5FA"/>
+        <bgColor rgb="FFFFF8E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -343,7 +383,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -388,6 +428,14 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -398,6 +446,14 @@
     </xf>
     <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="2" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -422,7 +478,7 @@
       <rgbColor rgb="FF800000"/>
       <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF4A6741"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFCCCCCC"/>
@@ -430,7 +486,7 @@
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FFA84055"/>
       <rgbColor rgb="FFFFF9E6"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFF0F5FA"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF1F5C8B"/>
@@ -462,11 +518,11 @@
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF0A0A0A"/>
-      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF1A1A1A"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF1A1A1A"/>
+      <rgbColor rgb="FF3A5A7A"/>
+      <rgbColor rgb="FF333333"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -652,7 +708,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
@@ -947,85 +1003,129 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B28" s="8" t="s">
+    <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C28" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="D28" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
+      <c r="B29" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="C29" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D29" s="12"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C30" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D30" s="6"/>
+      <c r="C30" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" s="10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B31" s="8" t="s">
         <v>35</v>
       </c>
       <c r="C31" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D31" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D31" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B32" s="8" t="s">
+      <c r="B33" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C32" s="9" t="s">
+      <c r="C33" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D33" s="6"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="D32" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="11" t="s">
+      <c r="B34" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="11"/>
-      <c r="C35" s="11"/>
-      <c r="D35" s="12" t="n">
-        <f aca="false">D6+D7+D10+D11+D12+D15+D16+D17+D20+D21+D22+D25+D26+D27+D28</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="13" t="s">
+      <c r="C34" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B36" s="13"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
+      <c r="D34" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D35" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B38" s="13"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="14" t="n">
+        <f aca="false">D6+D7+D10+D11+D12+D15+D16+D17+D20+D21+D22+D25+D26+D27+D30+D31</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B39" s="15"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="15"/>
+    </row>
+    <row r="41" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="16"/>
+      <c r="C41" s="16"/>
+      <c r="D41" s="16"/>
+    </row>
+    <row r="42" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B42" s="17"/>
+      <c r="C42" s="17"/>
+      <c r="D42" s="17"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="B42:D42"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1042,7 +1142,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
@@ -1053,7 +1153,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1337,85 +1437,129 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B28" s="8" t="s">
+    <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C28" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="D28" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
+      <c r="B29" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="C29" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D29" s="12"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C30" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D30" s="6"/>
+      <c r="C30" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" s="10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B31" s="8" t="s">
         <v>35</v>
       </c>
       <c r="C31" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D31" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D31" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B32" s="8" t="s">
+      <c r="B33" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C32" s="9" t="s">
+      <c r="C33" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D33" s="6"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="D32" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="11" t="s">
+      <c r="B34" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="11"/>
-      <c r="C35" s="11"/>
-      <c r="D35" s="12" t="n">
-        <f aca="false">D6+D7+D10+D11+D12+D15+D16+D17+D20+D21+D22+D25+D26+D27+D28</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="13" t="s">
+      <c r="C34" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B36" s="13"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
+      <c r="D34" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D35" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B38" s="13"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="14" t="n">
+        <f aca="false">D6+D7+D10+D11+D12+D15+D16+D17+D20+D21+D22+D25+D26+D27+D30+D31</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B39" s="15"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="15"/>
+    </row>
+    <row r="41" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="16"/>
+      <c r="C41" s="16"/>
+      <c r="D41" s="16"/>
+    </row>
+    <row r="42" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B42" s="17"/>
+      <c r="C42" s="17"/>
+      <c r="D42" s="17"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="B42:D42"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1432,7 +1576,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
@@ -1443,7 +1587,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1727,85 +1871,129 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B28" s="8" t="s">
+    <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C28" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="D28" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
+      <c r="B29" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="C29" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D29" s="12"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C30" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D30" s="6"/>
+      <c r="C30" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" s="10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B31" s="8" t="s">
         <v>35</v>
       </c>
       <c r="C31" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D31" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D31" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B32" s="8" t="s">
+      <c r="B33" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C32" s="9" t="s">
+      <c r="C33" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D33" s="6"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="D32" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="11" t="s">
+      <c r="B34" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="11"/>
-      <c r="C35" s="11"/>
-      <c r="D35" s="12" t="n">
-        <f aca="false">D6+D7+D10+D11+D12+D15+D16+D17+D20+D21+D22+D25+D26+D27+D28</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="13" t="s">
+      <c r="C34" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B36" s="13"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
+      <c r="D34" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D35" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B38" s="13"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="14" t="n">
+        <f aca="false">D6+D7+D10+D11+D12+D15+D16+D17+D20+D21+D22+D25+D26+D27+D30+D31</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B39" s="15"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="15"/>
+    </row>
+    <row r="41" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="16"/>
+      <c r="C41" s="16"/>
+      <c r="D41" s="16"/>
+    </row>
+    <row r="42" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B42" s="17"/>
+      <c r="C42" s="17"/>
+      <c r="D42" s="17"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="B42:D42"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1822,7 +2010,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
@@ -1833,7 +2021,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2117,85 +2305,129 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B28" s="8" t="s">
+    <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C28" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="D28" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
+      <c r="B29" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="C29" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D29" s="12"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C30" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D30" s="6"/>
+      <c r="C30" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" s="10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B31" s="8" t="s">
         <v>35</v>
       </c>
       <c r="C31" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D31" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D31" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B32" s="8" t="s">
+      <c r="B33" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C32" s="9" t="s">
+      <c r="C33" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D33" s="6"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="D32" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="11" t="s">
+      <c r="B34" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="11"/>
-      <c r="C35" s="11"/>
-      <c r="D35" s="12" t="n">
-        <f aca="false">D6+D7+D10+D11+D12+D15+D16+D17+D20+D21+D22+D25+D26+D27+D28</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="13" t="s">
+      <c r="C34" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B36" s="13"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
+      <c r="D34" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D35" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B38" s="13"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="14" t="n">
+        <f aca="false">D6+D7+D10+D11+D12+D15+D16+D17+D20+D21+D22+D25+D26+D27+D30+D31</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B39" s="15"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="15"/>
+    </row>
+    <row r="41" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="16"/>
+      <c r="C41" s="16"/>
+      <c r="D41" s="16"/>
+    </row>
+    <row r="42" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B42" s="17"/>
+      <c r="C42" s="17"/>
+      <c r="D42" s="17"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="B42:D42"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
feat: soporte INCLUIDO en precio — badge verde, excluye del total
</commit_message>
<xml_diff>
--- a/venuedata.xlsx
+++ b/venuedata.xlsx
@@ -424,7 +424,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1090,7 +1090,7 @@
       <c r="B38" s="13"/>
       <c r="C38" s="13"/>
       <c r="D38" s="14" t="n">
-        <f aca="false">D6+D7+D10+D11+D12+D15+D16+D17+D20+D21+D22+D25+D26+D27+D30+D31</f>
+        <f aca="false">IFERROR(D6,0)+IFERROR(D7,0)+IFERROR(D10,0)+IFERROR(D11,0)+IFERROR(D12,0)+IFERROR(D15,0)+IFERROR(D16,0)+IFERROR(D17,0)+IFERROR(D20,0)+IFERROR(D21,0)+IFERROR(D22,0)+IFERROR(D25,0)+IFERROR(D26,0)+IFERROR(D27,0)+IFERROR(D30,0)+IFERROR(D31,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -1524,7 +1524,7 @@
       <c r="B38" s="13"/>
       <c r="C38" s="13"/>
       <c r="D38" s="14" t="n">
-        <f aca="false">D6+D7+D10+D11+D12+D15+D16+D17+D20+D21+D22+D25+D26+D27+D30+D31</f>
+        <f aca="false">IFERROR(D6,0)+IFERROR(D7,0)+IFERROR(D10,0)+IFERROR(D11,0)+IFERROR(D12,0)+IFERROR(D15,0)+IFERROR(D16,0)+IFERROR(D17,0)+IFERROR(D20,0)+IFERROR(D21,0)+IFERROR(D22,0)+IFERROR(D25,0)+IFERROR(D26,0)+IFERROR(D27,0)+IFERROR(D30,0)+IFERROR(D31,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -1958,7 +1958,7 @@
       <c r="B38" s="13"/>
       <c r="C38" s="13"/>
       <c r="D38" s="14" t="n">
-        <f aca="false">D6+D7+D10+D11+D12+D15+D16+D17+D20+D21+D22+D25+D26+D27+D30+D31</f>
+        <f aca="false">IFERROR(D6,0)+IFERROR(D7,0)+IFERROR(D10,0)+IFERROR(D11,0)+IFERROR(D12,0)+IFERROR(D15,0)+IFERROR(D16,0)+IFERROR(D17,0)+IFERROR(D20,0)+IFERROR(D21,0)+IFERROR(D22,0)+IFERROR(D25,0)+IFERROR(D26,0)+IFERROR(D27,0)+IFERROR(D30,0)+IFERROR(D31,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2392,7 +2392,7 @@
       <c r="B38" s="13"/>
       <c r="C38" s="13"/>
       <c r="D38" s="14" t="n">
-        <f aca="false">D6+D7+D10+D11+D12+D15+D16+D17+D20+D21+D22+D25+D26+D27+D30+D31</f>
+        <f aca="false">IFERROR(D6,0)+IFERROR(D7,0)+IFERROR(D10,0)+IFERROR(D11,0)+IFERROR(D12,0)+IFERROR(D15,0)+IFERROR(D16,0)+IFERROR(D17,0)+IFERROR(D20,0)+IFERROR(D21,0)+IFERROR(D22,0)+IFERROR(D25,0)+IFERROR(D26,0)+IFERROR(D27,0)+IFERROR(D30,0)+IFERROR(D31,0)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>